<commit_message>
chore: update schedules 2026-08-28
</commit_message>
<xml_diff>
--- a/output/one_schedules_latest.xlsx
+++ b/output/one_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:M51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -518,7 +518,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -528,12 +528,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE</t>
+          <t>ATHENS BRIDGE</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE 186S</t>
+          <t>ATHENS BRIDGE 1188S</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -548,7 +548,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>56</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -558,7 +558,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -595,12 +595,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>ATHENS BRIDGE</t>
+          <t>EMMANUEL P</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>ATHENS BRIDGE 1188S</t>
+          <t>EMMANUEL P 013S</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-11-04</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -652,22 +652,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>SX1</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>EMMANUEL P</t>
+          <t>MSC SHUBA B</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>EMMANUEL P 013S</t>
+          <t>MSC SHUBA B FI635A</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -677,12 +677,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-11-04</t>
+          <t>2026-11-11</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>58</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -719,22 +719,22 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>MSC SHUBA B</t>
+          <t>NAVIOS CHRYSALIS</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>MSC SHUBA B FI635A</t>
+          <t>NAVIOS CHRYSALIS 017S</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -744,12 +744,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-11-04</t>
+          <t>2026-11-11</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>56</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -759,7 +759,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -786,22 +786,22 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>SX1</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS</t>
+          <t>MSC AVNI</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS 017S</t>
+          <t>MSC AVNI FI636A</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>53</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -853,22 +853,22 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>MSC AVNI</t>
+          <t>NAVIOS VERDE</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>MSC AVNI FI636A</t>
+          <t>NAVIOS VERDE 187S</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -878,12 +878,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-11-11</t>
+          <t>2026-11-18</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>56</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -893,14 +893,14 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HKHKG→SEGOT</t>
+          <t>HKHKG→NOOSL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -910,7 +910,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SEGOT</t>
+          <t>NOOSL</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -930,27 +930,27 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE</t>
+          <t>ATHENS BRIDGE</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE 187S</t>
+          <t>ATHENS BRIDGE 1188S</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>GOTHENBURG</t>
+          <t>ROTTERDAM</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-11-18</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>49</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -987,7 +987,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -997,12 +997,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE</t>
+          <t>ATHENS BRIDGE</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE 186S</t>
+          <t>ATHENS BRIDGE 1188S</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1012,12 +1012,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1064,12 +1064,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE</t>
+          <t>EMMANUEL P</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE 186S</t>
+          <t>EMMANUEL P 013S</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1079,12 +1079,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>49</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1131,12 +1131,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>ATHENS BRIDGE</t>
+          <t>EMMANUEL P</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>ATHENS BRIDGE 1188S</t>
+          <t>EMMANUEL P 013S</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1146,12 +1146,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>56</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1188,22 +1188,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>SX1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>ATHENS BRIDGE</t>
+          <t>MSC SHUBA B</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>ATHENS BRIDGE 1188S</t>
+          <t>MSC SHUBA B FI635A</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1213,12 +1213,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>51</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1265,12 +1265,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>EMMANUEL P</t>
+          <t>NAVIOS CHRYSALIS</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>EMMANUEL P 013S</t>
+          <t>NAVIOS CHRYSALIS 017S</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1332,12 +1332,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>EMMANUEL P</t>
+          <t>NAVIOS CHRYSALIS</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>EMMANUEL P 013S</t>
+          <t>NAVIOS CHRYSALIS 017S</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>49</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1399,12 +1399,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>MSC SHUBA B</t>
+          <t>MSC AVNI</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>MSC SHUBA B FI635A</t>
+          <t>MSC AVNI FI636A</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1414,12 +1414,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>46</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1466,12 +1466,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS</t>
+          <t>NAVIOS VERDE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS 017S</t>
+          <t>NAVIOS VERDE 187S</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1523,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1533,12 +1533,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS</t>
+          <t>NAVIOS VERDE</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS 017S</t>
+          <t>NAVIOS VERDE 187S</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1548,7 +1548,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-11-06</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1563,49 +1563,45 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HKHKG→NOOSL</t>
+          <t>VNSGN→NOTAE</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>NOOSL</t>
+          <t>NOTAE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>HONG KONG</t>
+          <t>CAI MEP</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>SX1</t>
-        </is>
-      </c>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>MSC AVNI</t>
+          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>MSC AVNI FI636A</t>
+          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1615,12 +1611,12 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>43</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1630,49 +1626,45 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>HKHKG→NOOSL</t>
+          <t>VNSGN→NOTAE</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>NOOSL</t>
+          <t>NOTAE</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>HONG KONG</t>
+          <t>CAI MEP</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>JSM</t>
-        </is>
-      </c>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE</t>
+          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE 187S</t>
+          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1682,64 +1674,60 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>55</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (2)</t>
+          <t>TRANSSHIPMENT (3)</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>HKHKG→NOOSL</t>
+          <t>VNSGN→NOTAE</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>NOOSL</t>
+          <t>NOTAE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>HONG KONG</t>
+          <t>CAI MEP</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>JSM</t>
-        </is>
-      </c>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE</t>
+          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE 187S</t>
+          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1749,22 +1737,22 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>53</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (2)</t>
+          <t>TRANSSHIPMENT (3)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1779,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1812,12 +1800,12 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>42</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1827,7 +1815,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1842,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -1875,22 +1863,22 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>42</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (3)</t>
+          <t>TRANSSHIPMENT (2)</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -1917,7 +1905,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -1938,274 +1926,290 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>43</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (3)</t>
+          <t>TRANSSHIPMENT (2)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>VNSGN→NOTAE</t>
+          <t>CNTAO→ITSPE</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>CNTAO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>NOTAE</t>
+          <t>ITSPE</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>CAI MEP</t>
+          <t>QINGDAO, SHANDONG</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>PN3</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
+          <t>HMM VANCOUVER</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
+          <t>HMM VANCOUVER 307E</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>ROTTERDAM</t>
+          <t>LA SPEZIA</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-11-12</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>75</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (2)</t>
+          <t>TRANSSHIPMENT (1)</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>VNSGN→NOTAE</t>
+          <t>CNTAO→ITSPE</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>CNTAO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>NOTAE</t>
+          <t>ITSPE</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>CAI MEP</t>
+          <t>QINGDAO, SHANDONG</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>FE3</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
+          <t>ONE FOREVER</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
+          <t>ONE FOREVER 010W</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>ROTTERDAM</t>
+          <t>LA SPEZIA</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>58</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (2)</t>
+          <t>TRANSSHIPMENT (1)</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>VNSGN→NOTAE</t>
+          <t>CNTAO→ITSPE</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>CNTAO</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>NOTAE</t>
+          <t>ITSPE</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>CAI MEP</t>
+          <t>QINGDAO, SHANDONG</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>FE3</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
+          <t>ONE FOREVER</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
+          <t>ONE FOREVER 010W</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>ROTTERDAM</t>
+          <t>LA SPEZIA</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>68</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (3)</t>
+          <t>TRANSSHIPMENT (1)</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>VNSGN→NOTAE</t>
+          <t>CNTAO→ITSPE</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>CNTAO</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>NOTAE</t>
+          <t>ITSPE</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>CAI MEP</t>
+          <t>QINGDAO, SHANDONG</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>AX3</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
+          <t>YOKOHAMA EXPRESS</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
+          <t>YOKOHAMA EXPRESS 2634E</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>ROTTERDAM</t>
+          <t>LA SPEZIA</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>66</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (2)</t>
+          <t>TRANSSHIPMENT (1)</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2236,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2242,12 +2246,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>HMM VANCOUVER</t>
+          <t>HYUNDAI SUPREME</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>HMM VANCOUVER 307E</t>
+          <t>HYUNDAI SUPREME 159E</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2257,12 +2261,12 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>79</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2272,7 +2276,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2299,22 +2303,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>AX4</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>ONE FOREVER</t>
+          <t>CONTI CONTESSA</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>ONE FOREVER 010W</t>
+          <t>CONTI CONTESSA 026E</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2324,12 +2328,12 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>65</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -2339,7 +2343,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2366,22 +2370,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>AX4</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>ONE FOREVER</t>
+          <t>ONE COMPETENCE</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>ONE FOREVER 010W</t>
+          <t>ONE COMPETENCE 099E</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2391,12 +2395,12 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
+          <t>2026-11-12</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>70</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -2406,7 +2410,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2433,7 +2437,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2443,12 +2447,12 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>YOKOHAMA EXPRESS</t>
+          <t>POSORJA EXPRESS</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>YOKOHAMA EXPRESS 2634E</t>
+          <t>POSORJA EXPRESS 2633E</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2458,12 +2462,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
+          <t>2026-11-12</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>68</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -2473,7 +2477,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2500,22 +2504,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>PN3</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>HYUNDAI SUPREME</t>
+          <t>HMM COPENHAGEN</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>HYUNDAI SUPREME 159E</t>
+          <t>HMM COPENHAGEN 020W</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2525,12 +2529,12 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-02</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>79</t>
+          <t>58</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -2540,7 +2544,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2567,22 +2571,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>AX4</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>CONTI CONTESSA</t>
+          <t>HMM COPENHAGEN</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>CONTI CONTESSA 026E</t>
+          <t>HMM COPENHAGEN 020W</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2597,7 +2601,7 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>61</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -2607,7 +2611,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2634,22 +2638,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>AX3</t>
+          <t>AX4</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>POSORJA EXPRESS</t>
+          <t>HYUNDAI COURAGE</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>POSORJA EXPRESS 2633E</t>
+          <t>HYUNDAI COURAGE 125E</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2659,7 +2663,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -2674,7 +2678,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2701,22 +2705,22 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>AX4</t>
+          <t>LAW</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>ONE COMPETENCE</t>
+          <t>HMM OAKLAND</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>ONE COMPETENCE 099E</t>
+          <t>HMM OAKLAND 140E</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2726,7 +2730,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -2741,7 +2745,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2768,22 +2772,22 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>CTP</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>HMM COPENHAGEN</t>
+          <t>ACX PEARL</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>HMM COPENHAGEN 020W</t>
+          <t>ACX PEARL 0291S</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2793,12 +2797,12 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-11-02</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>68</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -2808,7 +2812,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2835,22 +2839,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>IAE</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>HMM COPENHAGEN</t>
+          <t>MARIA C</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>HMM COPENHAGEN 020W</t>
+          <t>MARIA C 197E</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2860,12 +2864,12 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-11-05</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>68</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -2875,7 +2879,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2902,22 +2906,22 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>AX4</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>HYUNDAI COURAGE</t>
+          <t>HMM ST PETERSBURG</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>HYUNDAI COURAGE 125E</t>
+          <t>HMM ST PETERSBURG 019W</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2927,12 +2931,12 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>57</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -2942,7 +2946,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -2969,22 +2973,22 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>LAW</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>HMM OAKLAND</t>
+          <t>HMM ST PETERSBURG</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>HMM OAKLAND 140E</t>
+          <t>HMM ST PETERSBURG 019W</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2999,7 +3003,7 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>59</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -3009,7 +3013,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -3036,22 +3040,22 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>CTP</t>
+          <t>PN3</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>ACX PEARL</t>
+          <t>ONE DURBAN</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>ACX PEARL 0291S</t>
+          <t>ONE DURBAN 001E</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3061,12 +3065,12 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>80</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -3076,7 +3080,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -3103,22 +3107,22 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>IAE</t>
+          <t>AX3</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>MARIA C</t>
+          <t>IQUIQUE EXPRESS</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>MARIA C 197E</t>
+          <t>IQUIQUE EXPRESS 2636E</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3128,12 +3132,12 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>80</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -3143,7 +3147,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -3170,22 +3174,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>PN3</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>HMM ST PETERSBURG</t>
+          <t>YM WEALTH</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>HMM ST PETERSBURG 019W</t>
+          <t>YM WEALTH 193E</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3195,12 +3199,12 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-11-10</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>77</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -3210,7 +3214,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -3237,22 +3241,22 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>IAE</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>HMM ST PETERSBURG</t>
+          <t>MARIA C</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>HMM ST PETERSBURG 019W</t>
+          <t>MARIA C 198E</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3262,12 +3266,12 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>76</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -3277,7 +3281,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -3304,22 +3308,22 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>PN3</t>
+          <t>CTP</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>ONE DURBAN</t>
+          <t>BRIGHT SAKURA</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>ONE DURBAN 001E</t>
+          <t>BRIGHT SAKURA 0021S</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3334,7 +3338,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>75</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3344,7 +3348,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -3371,22 +3375,22 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>AX3</t>
+          <t>IAE</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>IQUIQUE EXPRESS</t>
+          <t>ONE DIAMOND</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>IQUIQUE EXPRESS 2636E</t>
+          <t>ONE DIAMOND 004E</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3401,7 +3405,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>80</t>
+          <t>75</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -3411,7 +3415,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -3438,22 +3442,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>PN3</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>YM WEALTH</t>
+          <t>HMM ROTTERDAM</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>YM WEALTH 193E</t>
+          <t>HMM ROTTERDAM 020W</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3463,12 +3467,12 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-11-10</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>51</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -3478,7 +3482,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -3505,22 +3509,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>IAE</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>MARIA C</t>
+          <t>HMM ROTTERDAM</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>MARIA C 198E</t>
+          <t>HMM ROTTERDAM 020W</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3530,12 +3534,12 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>60</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -3545,7 +3549,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -3572,22 +3576,22 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>CTP</t>
+          <t>AX4</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>BRIGHT SAKURA</t>
+          <t>SAPPHIRE TOWER</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>BRIGHT SAKURA 0021S</t>
+          <t>SAPPHIRE TOWER 005E</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3602,7 +3606,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>72</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -3612,7 +3616,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -3639,22 +3643,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>IAE</t>
+          <t>PN3</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>ONE DIAMOND</t>
+          <t>YM COSMOS</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>ONE DIAMOND 004E</t>
+          <t>YM COSMOS 192E</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3664,12 +3668,12 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-12-17</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>84</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -3679,7 +3683,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -3706,22 +3710,22 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>AX3</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>HMM ROTTERDAM</t>
+          <t>ONE SPARKLE</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>HMM ROTTERDAM 020W</t>
+          <t>ONE SPARKLE 2637E</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3731,12 +3735,12 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-11-10</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>69</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
@@ -3746,7 +3750,7 @@
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>
@@ -3773,22 +3777,22 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>IAE</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>HMM ROTTERDAM</t>
+          <t>ONE DIAMOND</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>HMM ROTTERDAM 020W</t>
+          <t>ONE DIAMOND 005E</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -3798,12 +3802,12 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>69</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
@@ -3813,141 +3817,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>2026-08-27 07:46 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>CNTAO→ITSPE</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>CNTAO</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>ITSPE</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>QINGDAO, SHANDONG</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>2026-09-22</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>AX4</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>SAPPHIRE TOWER</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>SAPPHIRE TOWER 005E</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>LA SPEZIA</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>2026-12-03</t>
-        </is>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>72</t>
-        </is>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>TRANSSHIPMENT (1)</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>2026-08-27 07:46 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>CNTAO→ITSPE</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>CNTAO</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>ITSPE</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>QINGDAO, SHANDONG</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>PN3</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>YM COSMOS</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>YM COSMOS 192E</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>LA SPEZIA</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr">
-        <is>
-          <t>2026-12-17</t>
-        </is>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>TRANSSHIPMENT (1)</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>2026-08-27 07:46 UTC</t>
+          <t>2026-08-28 09:51 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-09-05
</commit_message>
<xml_diff>
--- a/output/one_schedules_latest.xlsx
+++ b/output/one_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,7 +558,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1563,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>2026-09-04 03:10 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1800,12 +1800,12 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>48</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1815,7 +1815,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1878,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2031,22 +2031,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>AX3</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>HMM COPENHAGEN</t>
+          <t>POSORJA EXPRESS</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>HMM COPENHAGEN 020W</t>
+          <t>POSORJA EXPRESS 2633E</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2056,12 +2056,12 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>74</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2098,22 +2098,22 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>LAW</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>HMM COPENHAGEN</t>
+          <t>HMM OAKLAND</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>HMM COPENHAGEN 020W</t>
+          <t>HMM OAKLAND 140E</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2123,12 +2123,12 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>68</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2165,22 +2165,22 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>AX3</t>
+          <t>CTP</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>POSORJA EXPRESS</t>
+          <t>ACX PEARL</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>POSORJA EXPRESS 2633E</t>
+          <t>ACX PEARL 0291S</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2190,7 +2190,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2205,7 +2205,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2232,22 +2232,22 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>LAW</t>
+          <t>AX4</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>HMM OAKLAND</t>
+          <t>HYUNDAI COURAGE</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>HMM OAKLAND 140E</t>
+          <t>HYUNDAI COURAGE 125E</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>66</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2299,22 +2299,22 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>CTP</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>ACX PEARL</t>
+          <t>HMM ST PETERSBURG</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>ACX PEARL 0291S</t>
+          <t>HMM ST PETERSBURG 019W</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2324,12 +2324,12 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>56</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2371,17 +2371,17 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>AX4</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>HYUNDAI COURAGE</t>
+          <t>HMM ST PETERSBURG</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>HYUNDAI COURAGE 125E</t>
+          <t>HMM ST PETERSBURG 019W</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2438,17 +2438,17 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>IAE</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>HMM ST PETERSBURG</t>
+          <t>MARIA C</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>HMM ST PETERSBURG 019W</t>
+          <t>MARIA C 197E</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2458,12 +2458,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>66</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2500,22 +2500,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>AX3</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>HMM ST PETERSBURG</t>
+          <t>IQUIQUE EXPRESS</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>HMM ST PETERSBURG 019W</t>
+          <t>IQUIQUE EXPRESS 2636E</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2525,12 +2525,12 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>77</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -2540,7 +2540,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2567,22 +2567,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>IAE</t>
+          <t>PN3</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>MARIA C</t>
+          <t>YM WEALTH</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>MARIA C 197E</t>
+          <t>YM WEALTH 193E</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2592,12 +2592,12 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>77</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -2607,7 +2607,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2634,22 +2634,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>AX3</t>
+          <t>CTP</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>IQUIQUE EXPRESS</t>
+          <t>BRIGHT SAKURA</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>IQUIQUE EXPRESS 2636E</t>
+          <t>BRIGHT SAKURA 0021S</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2664,7 +2664,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>75</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2701,22 +2701,22 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>PN3</t>
+          <t>IAE</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>YM WEALTH</t>
+          <t>MARIA C</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>YM WEALTH 193E</t>
+          <t>MARIA C 198E</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>74</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2768,22 +2768,22 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>CTP</t>
+          <t>AX4</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>BRIGHT SAKURA</t>
+          <t>SAPPHIRE TOWER</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>BRIGHT SAKURA 0021S</t>
+          <t>SAPPHIRE TOWER 005E</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2798,7 +2798,7 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>74</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2840,17 +2840,17 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>IAE</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>MARIA C</t>
+          <t>HMM ROTTERDAM</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>MARIA C 198E</t>
+          <t>HMM ROTTERDAM 020W</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2860,12 +2860,12 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>57</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -2875,7 +2875,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2907,17 +2907,17 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>AX4</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>SAPPHIRE TOWER</t>
+          <t>HMM ROTTERDAM</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>SAPPHIRE TOWER 005E</t>
+          <t>HMM ROTTERDAM 020W</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2927,12 +2927,12 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>60</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -2969,22 +2969,22 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>PN3</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>HMM ROTTERDAM</t>
+          <t>ONE DURBAN</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>HMM ROTTERDAM 020W</t>
+          <t>ONE DURBAN 001E</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2994,12 +2994,12 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>71</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -3036,22 +3036,22 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>IAE</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>HMM ROTTERDAM</t>
+          <t>ONE DIAMOND</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>HMM ROTTERDAM 020W</t>
+          <t>ONE DIAMOND 004E</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3061,12 +3061,12 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>71</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -3103,22 +3103,22 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>PN3</t>
+          <t>AX3</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>ONE DURBAN</t>
+          <t>ONE SPARKLE</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>ONE DURBAN 001E</t>
+          <t>ONE SPARKLE 2637E</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>68</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -3170,22 +3170,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>IAE</t>
+          <t>AX4</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>ONE DIAMOND</t>
+          <t>EMERALD TOWER</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>ONE DIAMOND 004E</t>
+          <t>EMERALD TOWER 005E</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>67</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -3237,22 +3237,22 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>AX3</t>
+          <t>IAE</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>ONE SPARKLE</t>
+          <t>MARIA C</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>ONE SPARKLE 2637E</t>
+          <t>MARIA C 199E</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>66</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -3277,7 +3277,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -3304,22 +3304,22 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>AX4</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>EMERALD TOWER</t>
+          <t>HMM DRIVE</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>EMERALD TOWER 005E</t>
+          <t>HMM DRIVE 061W</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3329,12 +3329,12 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>49</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -3376,17 +3376,17 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>IAE</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>MARIA C</t>
+          <t>HMM DRIVE</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>MARIA C 199E</t>
+          <t>HMM DRIVE 061W</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -3443,17 +3443,17 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>AX3</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>HMM DRIVE</t>
+          <t>ONE SHINE</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>HMM DRIVE 061W</t>
+          <t>ONE SHINE 2638E</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3463,12 +3463,12 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-11-23</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>66</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -3478,7 +3478,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -3505,22 +3505,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>IAE</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>HMM DRIVE</t>
+          <t>ONE DIAMOND</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>HMM DRIVE 061W</t>
+          <t>ONE DIAMOND 005E</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>65</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>
@@ -3572,22 +3572,22 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-10-03</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>AX3</t>
+          <t>CTP</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>ONE SHINE</t>
+          <t>WAN HAI 331</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>ONE SHINE 2638E</t>
+          <t>WAN HAI 331 0030S</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3597,12 +3597,12 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-12-17</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>75</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -3612,74 +3612,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>2026-09-04 03:11 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>CNTAO→ITSPE</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>CNTAO</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>ITSPE</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>QINGDAO, SHANDONG</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>IAE</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>ONE DIAMOND</t>
-        </is>
-      </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>ONE DIAMOND 005E</t>
-        </is>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>LA SPEZIA</t>
-        </is>
-      </c>
-      <c r="J49" t="inlineStr">
-        <is>
-          <t>2026-12-03</t>
-        </is>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>65</t>
-        </is>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>TRANSSHIPMENT (1)</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>2026-09-04 03:11 UTC</t>
+          <t>2026-09-05 03:11 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-09-09
</commit_message>
<xml_diff>
--- a/output/one_schedules_latest.xlsx
+++ b/output/one_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M50"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,7 +558,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-08 03:17 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -585,22 +585,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>SX1</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS</t>
+          <t>MSC SHUBA B</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS 017S</t>
+          <t>MSC SHUBA B FI635A</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>58</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2026-09-08 03:17 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -652,22 +652,22 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>MSC SHUBA B</t>
+          <t>NAVIOS CHRYSALIS</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>MSC SHUBA B FI635A</t>
+          <t>NAVIOS CHRYSALIS 017S</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -682,7 +682,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>57</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -692,7 +692,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-08 03:17 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>2026-09-08 03:17 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -826,7 +826,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-09-08 03:17 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-08 03:17 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,14 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-08 03:17 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HKHKG→NOOSL</t>
+          <t>HKHKG→SEGOT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>NOOSL</t>
+          <t>SEGOT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1002,22 +1002,22 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>EMMANUEL P 013S</t>
+          <t>EMMANUEL P 014S</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>ROTTERDAM</t>
+          <t>GOTHENBURG</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-12-02</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>56</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1079,12 +1079,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>48</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1131,12 +1131,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS</t>
+          <t>EMMANUEL P</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS 017S</t>
+          <t>EMMANUEL P 013S</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>55</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1161,7 +1161,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1188,22 +1188,22 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>SX1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS</t>
+          <t>MSC SHUBA B</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>NAVIOS CHRYSALIS 017S</t>
+          <t>MSC SHUBA B FI635A</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1213,12 +1213,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>53</t>
+          <t>50</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1255,22 +1255,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>MSC SHUBA B</t>
+          <t>NAVIOS CHRYSALIS</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>MSC SHUBA B FI635A</t>
+          <t>NAVIOS CHRYSALIS 017S</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1280,12 +1280,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>43</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1332,12 +1332,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE</t>
+          <t>NAVIOS CHRYSALIS</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>NAVIOS VERDE 187S</t>
+          <t>NAVIOS CHRYSALIS 017S</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1414,12 +1414,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>48</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1456,22 +1456,22 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>MSC AVNI</t>
+          <t>NAVIOS VERDE</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>MSC AVNI FI636A</t>
+          <t>NAVIOS VERDE 187S</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1523,22 +1523,22 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>JSM</t>
+          <t>SX1</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>ATHENS BRIDGE</t>
+          <t>MSC AVNI</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>ATHENS BRIDGE 1189S</t>
+          <t>MSC AVNI FI636A</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1548,12 +1548,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>47</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1615,12 +1615,12 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-11-20</t>
+          <t>2026-11-12</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>48</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1657,22 +1657,22 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>SX1</t>
+          <t>JSM</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>PARANA EXPRESS</t>
+          <t>ATHENS BRIDGE</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>PARANA EXPRESS 2638W</t>
+          <t>ATHENS BRIDGE 1189S</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1682,12 +1682,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-20</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>56</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
@@ -1697,45 +1697,49 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>VNSGN→NOTAE</t>
+          <t>HKHKG→NOOSL</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>HKHKG</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>NOTAE</t>
+          <t>NOOSL</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>CAI MEP</t>
+          <t>HONG KONG</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
+          <t>2026-10-05</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>SX1</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
+          <t>PARANA EXPRESS</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
+          <t>PARANA EXPRESS 2638W</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1745,60 +1749,64 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>50</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (3)</t>
+          <t>TRANSSHIPMENT (2)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>VNSGN→NOTAE</t>
+          <t>HKHKG→NOOSL</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>HKHKG</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>NOTAE</t>
+          <t>NOOSL</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>CAI MEP</t>
+          <t>HONG KONG</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr"/>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>JSM</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
+          <t>EMMANUEL P</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
+          <t>EMMANUEL P 014S</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1808,12 +1816,12 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>48</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -1823,45 +1831,49 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>VNSGN→NOTAE</t>
+          <t>HKHKG→NOOSL</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>HKHKG</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>NOTAE</t>
+          <t>NOOSL</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>CAI MEP</t>
+          <t>HONG KONG</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>JSM</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
+          <t>EMMANUEL P</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
+          <t>EMMANUEL P 014S</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1871,22 +1883,22 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-11-20</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>49</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (3)</t>
+          <t>TRANSSHIPMENT (2)</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1913,7 +1925,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -1934,22 +1946,22 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>45</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (2)</t>
+          <t>TRANSSHIPMENT (3)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1988,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
@@ -1997,12 +2009,12 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>41</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -2012,7 +2024,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2039,7 +2051,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -2060,12 +2072,12 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>48</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -2075,7 +2087,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2114,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -2123,12 +2135,12 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-11-06</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>43</t>
+          <t>41</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -2138,208 +2150,196 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CNTAO→ITSPE</t>
+          <t>VNSGN→NOTAE</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CNTAO</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ITSPE</t>
+          <t>NOTAE</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>QINGDAO, SHANDONG</t>
+          <t>CAI MEP</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>LAW</t>
-        </is>
-      </c>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
-          <t>HMM OAKLAND</t>
+          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>HMM OAKLAND 140E</t>
+          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>LA SPEZIA</t>
+          <t>ROTTERDAM</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>43</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (1)</t>
+          <t>TRANSSHIPMENT (2)</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CNTAO→ITSPE</t>
+          <t>VNSGN→NOTAE</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CNTAO</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>ITSPE</t>
+          <t>NOTAE</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>QINGDAO, SHANDONG</t>
+          <t>CAI MEP</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>AX4</t>
-        </is>
-      </c>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
-          <t>HYUNDAI COURAGE</t>
+          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>HYUNDAI COURAGE 125E</t>
+          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>LA SPEZIA</t>
+          <t>ROTTERDAM</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>48</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (1)</t>
+          <t>TRANSSHIPMENT (3)</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CNTAO→ITSPE</t>
+          <t>VNSGN→NOTAE</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CNTAO</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>ITSPE</t>
+          <t>NOTAE</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>QINGDAO, SHANDONG</t>
+          <t>CAI MEP</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>CTP</t>
-        </is>
-      </c>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
-          <t>ACX PEARL</t>
+          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>ACX PEARL 0291S</t>
+          <t>CONG TY TNHH CANG QUOC TE TAN CANG CAI MEP (WATER)</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>LA SPEZIA</t>
+          <t>ROTTERDAM</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-11-05</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>42</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>TRANSSHIPMENT (1)</t>
+          <t>TRANSSHIPMENT (2)</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:20 UTC</t>
         </is>
       </c>
     </row>
@@ -2366,22 +2366,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>LAW</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>HMM ST PETERSBURG</t>
+          <t>HMM OAKLAND</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>HMM ST PETERSBURG 019W</t>
+          <t>HMM OAKLAND 140E</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2391,12 +2391,12 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-11-09</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>68</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -2438,17 +2438,17 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>AX4</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>HMM ST PETERSBURG</t>
+          <t>HYUNDAI COURAGE</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>HMM ST PETERSBURG 019W</t>
+          <t>HYUNDAI COURAGE 125E</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -2458,12 +2458,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>66</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -2473,7 +2473,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -2500,22 +2500,22 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>IAE</t>
+          <t>CTP</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>MARIA C</t>
+          <t>ACX PEARL</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>MARIA C 197E</t>
+          <t>ACX PEARL 0291S</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>66</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -2540,7 +2540,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -2567,22 +2567,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>AX3</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>IQUIQUE EXPRESS</t>
+          <t>HMM ST PETERSBURG</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>IQUIQUE EXPRESS 2636E</t>
+          <t>HMM ST PETERSBURG 019W</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2592,12 +2592,12 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-11-09</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>56</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -2607,7 +2607,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -2634,22 +2634,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>PN3</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>YM WEALTH</t>
+          <t>HMM ST PETERSBURG</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>YM WEALTH 193E</t>
+          <t>HMM ST PETERSBURG 019W</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2659,12 +2659,12 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-11-12</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>59</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -2701,22 +2701,22 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>CTP</t>
+          <t>IAE</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>BRIGHT SAKURA</t>
+          <t>MARIA C</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>BRIGHT SAKURA 0021S</t>
+          <t>MARIA C 197E</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2726,12 +2726,12 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>65</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -2768,22 +2768,22 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>PN3</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>HMM ROTTERDAM</t>
+          <t>YM WEALTH</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>HMM ROTTERDAM 020W</t>
+          <t>YM WEALTH 193E</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2793,12 +2793,12 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>77</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -2835,22 +2835,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>AX3</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>HMM ROTTERDAM</t>
+          <t>IQUIQUE EXPRESS</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>HMM ROTTERDAM 020W</t>
+          <t>IQUIQUE EXPRESS 2636E</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2860,12 +2860,12 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-11-19</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>76</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -2875,7 +2875,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -2902,22 +2902,22 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>IAE</t>
+          <t>CTP</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>MARIA C</t>
+          <t>BRIGHT SAKURA</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>MARIA C 198E</t>
+          <t>BRIGHT SAKURA 0021S</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>75</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -2969,22 +2969,22 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>AX4</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>SAPPHIRE TOWER</t>
+          <t>HMM ROTTERDAM</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>SAPPHIRE TOWER 005E</t>
+          <t>HMM ROTTERDAM 020W</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -2994,12 +2994,12 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>57</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -3009,7 +3009,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3036,22 +3036,22 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>PN3</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>ONE DURBAN</t>
+          <t>HMM ROTTERDAM</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>ONE DURBAN 001E</t>
+          <t>HMM ROTTERDAM 020W</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3061,12 +3061,12 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-11-19</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>60</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -3076,7 +3076,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3103,7 +3103,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3113,12 +3113,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>ONE DIAMOND</t>
+          <t>MARIA C</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>ONE DIAMOND 004E</t>
+          <t>MARIA C 198E</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>73</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3170,22 +3170,22 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>AX3</t>
+          <t>PN3</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>ONE SPARKLE</t>
+          <t>ONE DURBAN</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>ONE SPARKLE 2637E</t>
+          <t>ONE DURBAN 001E</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>72</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -3210,7 +3210,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3237,22 +3237,22 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>IAE</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>HMM DRIVE</t>
+          <t>ONE DIAMOND</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>HMM DRIVE 061W</t>
+          <t>ONE DIAMOND 004E</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3262,12 +3262,12 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>71</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -3277,7 +3277,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3304,22 +3304,22 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>FE3</t>
+          <t>AX3</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>HMM DRIVE</t>
+          <t>ONE SPARKLE</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>HMM DRIVE 061W</t>
+          <t>ONE SPARKLE 2637E</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3334,7 +3334,7 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>68</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3381,12 +3381,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>EMERALD TOWER</t>
+          <t>SAPPHIRE TOWER</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>EMERALD TOWER 005E</t>
+          <t>SAPPHIRE TOWER 005E</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>68</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
@@ -3411,7 +3411,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3443,17 +3443,17 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>IAE</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>MARIA C</t>
+          <t>HMM DRIVE</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>MARIA C 199E</t>
+          <t>HMM DRIVE 061W</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -3463,12 +3463,12 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-12-03</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>49</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
@@ -3478,7 +3478,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3510,17 +3510,17 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>AX3</t>
+          <t>FE3</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>ONE SHINE</t>
+          <t>HMM DRIVE</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>ONE SHINE 2638E</t>
+          <t>HMM DRIVE 061W</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3572,22 +3572,22 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>IAE</t>
+          <t>AX4</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>ONE DIAMOND</t>
+          <t>EMERALD TOWER</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>ONE DIAMOND 005E</t>
+          <t>EMERALD TOWER 005E</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3602,7 +3602,7 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>65</t>
+          <t>66</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3639,22 +3639,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-10-04</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>CTP</t>
+          <t>AX3</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>WAN HAI 331</t>
+          <t>ONE SHINE</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>WAN HAI 331 0030S</t>
+          <t>ONE SHINE 2638E</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -3664,12 +3664,12 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-12-17</t>
+          <t>2026-12-03</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>66</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>2026-09-08 03:18 UTC</t>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3706,47 +3706,248 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>IAE</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>MARIA C</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>MARIA C 199E</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>LA SPEZIA</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-12-03</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>TRANSSHIPMENT (1)</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>2026-09-09 03:21 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>CNTAO→ITSPE</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>CNTAO</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>ITSPE</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>QINGDAO, SHANDONG</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>IAE</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>ONE DIAMOND</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>ONE DIAMOND 005E</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>LA SPEZIA</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-12-03</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>TRANSSHIPMENT (1)</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>2026-09-09 03:21 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CNTAO→ITSPE</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>CNTAO</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ITSPE</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>QINGDAO, SHANDONG</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
           <t>2026-10-04</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>CTP</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>WAN HAI 331</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>WAN HAI 331 0030S</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>LA SPEZIA</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-12-17</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>TRANSSHIPMENT (1)</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>2026-09-09 03:21 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>CNTAO→ITSPE</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>CNTAO</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>ITSPE</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>QINGDAO, SHANDONG</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
         <is>
           <t>AX4</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="G53" t="inlineStr">
         <is>
           <t>HYUNDAI BRAVE</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>HYUNDAI BRAVE 120E</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>LA SPEZIA</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="J53" t="inlineStr">
         <is>
           <t>2026-12-17</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
+      <c r="K53" t="inlineStr">
         <is>
           <t>74</t>
         </is>
       </c>
-      <c r="L50" t="inlineStr">
+      <c r="L53" t="inlineStr">
         <is>
           <t>TRANSSHIPMENT (1)</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>2026-09-08 03:18 UTC</t>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>2026-09-09 03:21 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>